<commit_message>
fix(order): forecast Excel adds IST and remaining forecast in the current month
'Gesamt' of the sheet 'Umsatz kumuliert' and of Planning_Data (the plan) took the
larger of IST and forecast in the current month; they now add both, as the charts
and the project overview do. The note on this in 'Grafiken 1' is removed.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projectforge-business/src/main/resources/officeTemplates/ForecastTemplate.xlsx
+++ b/projectforge-business/src/main/resources/officeTemplates/ForecastTemplate.xlsx
@@ -5460,93 +5460,6 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>469900</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Textfeld 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97D60B30-C0AF-E040-A430-75769E8C30E1}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9867900" y="25400"/>
-          <a:ext cx="4013200" cy="533400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Anmerkung:</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> Im aktuellen Monat wird der größere Wert verwendet: Die IST-Daten (Rechnungen) oder der Monatsforecast.</a:t>
-          </a:r>
-          <a:endParaRPr lang="de-DE" sz="1100">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7687,11 +7600,11 @@
         <v>27</v>
       </c>
       <c r="B4" s="18">
-        <f>MAX(B2,B3)</f>
+        <f>B2+B3</f>
         <v>0</v>
       </c>
       <c r="C4" s="18">
-        <f t="shared" ref="C4:M4" si="0">MAX(C2,C3)</f>
+        <f t="shared" ref="C4:M4" si="0">C2+C3</f>
         <v>0</v>
       </c>
       <c r="D4" s="18">
@@ -8830,11 +8743,11 @@
         <v>27</v>
       </c>
       <c r="AD7" s="16">
-        <f ca="1">MAX(SUM(AD2:AD6),AD8)</f>
+        <f ca="1">SUM(AD2:AD6)+AD8</f>
         <v>0</v>
       </c>
       <c r="AE7" s="16">
-        <f t="shared" ref="AE7:AO7" ca="1" si="5">MAX(SUM(AE2:AE6),AE8)</f>
+        <f t="shared" ref="AE7:AO7" ca="1" si="5">SUM(AE2:AE6)+AE8</f>
         <v>0</v>
       </c>
       <c r="AF7" s="16">

</xml_diff>